<commit_message>
feat: add Capacitor deep link handling and improve task status UI labels
</commit_message>
<xml_diff>
--- a/Tarefas.xlsx
+++ b/Tarefas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="90">
   <si>
     <t>nome</t>
   </si>
@@ -269,6 +269,18 @@
   </si>
   <si>
     <t>adicionar rascunho de tarefas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">terminar o questionário </t>
+  </si>
+  <si>
+    <t xml:space="preserve">preparar breve plano de aula </t>
+  </si>
+  <si>
+    <t>integração HUB-Processos</t>
+  </si>
+  <si>
+    <t>listas de cálculo</t>
   </si>
 </sst>
 </file>
@@ -1507,7 +1519,9 @@
       <c r="E32" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G32" s="8"/>
+      <c r="G32" s="17">
+        <v>46237.0</v>
+      </c>
       <c r="J32" s="6" t="s">
         <v>22</v>
       </c>
@@ -1551,7 +1565,9 @@
       <c r="E34" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G34" s="17"/>
+      <c r="G34" s="17">
+        <v>46237.0</v>
+      </c>
       <c r="J34" s="6" t="s">
         <v>22</v>
       </c>
@@ -1595,7 +1611,9 @@
       <c r="E36" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G36" s="8"/>
+      <c r="G36" s="17">
+        <v>46237.0</v>
+      </c>
       <c r="J36" s="6" t="s">
         <v>22</v>
       </c>
@@ -1639,7 +1657,9 @@
       <c r="E38" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G38" s="8"/>
+      <c r="G38" s="17">
+        <v>46237.0</v>
+      </c>
       <c r="H38" s="9" t="s">
         <v>71</v>
       </c>
@@ -1708,7 +1728,9 @@
       <c r="E41" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G41" s="8"/>
+      <c r="G41" s="17">
+        <v>46230.0</v>
+      </c>
       <c r="J41" s="6" t="s">
         <v>22</v>
       </c>
@@ -1730,7 +1752,9 @@
       <c r="E42" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G42" s="17"/>
+      <c r="G42" s="17">
+        <v>46222.0</v>
+      </c>
       <c r="J42" s="6" t="s">
         <v>22</v>
       </c>
@@ -1752,7 +1776,9 @@
       <c r="E43" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G43" s="8"/>
+      <c r="G43" s="17">
+        <v>46222.0</v>
+      </c>
       <c r="J43" s="6" t="s">
         <v>22</v>
       </c>
@@ -1931,38 +1957,58 @@
       <c r="K51" s="10"/>
     </row>
     <row r="52" ht="22.5" customHeight="1">
+      <c r="A52" s="9" t="s">
+        <v>86</v>
+      </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="20"/>
       <c r="E52" s="20"/>
-      <c r="G52" s="8"/>
+      <c r="G52" s="17">
+        <v>46223.0</v>
+      </c>
       <c r="J52" s="10"/>
       <c r="K52" s="10"/>
     </row>
     <row r="53" ht="22.5" customHeight="1">
+      <c r="A53" s="9" t="s">
+        <v>87</v>
+      </c>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
       <c r="D53" s="20"/>
       <c r="E53" s="20"/>
-      <c r="G53" s="8"/>
+      <c r="G53" s="17">
+        <v>46224.0</v>
+      </c>
       <c r="J53" s="10"/>
       <c r="K53" s="10"/>
     </row>
     <row r="54" ht="22.5" customHeight="1">
+      <c r="A54" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
       <c r="D54" s="20"/>
       <c r="E54" s="20"/>
-      <c r="G54" s="8"/>
+      <c r="G54" s="17">
+        <v>46224.0</v>
+      </c>
       <c r="J54" s="10"/>
       <c r="K54" s="10"/>
     </row>
     <row r="55" ht="22.5" customHeight="1">
+      <c r="A55" s="9" t="s">
+        <v>89</v>
+      </c>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
       <c r="D55" s="7"/>
       <c r="E55" s="20"/>
-      <c r="G55" s="8"/>
+      <c r="G55" s="17">
+        <v>46225.0</v>
+      </c>
       <c r="J55" s="10"/>
       <c r="K55" s="10"/>
     </row>

</xml_diff>